<commit_message>
Streamlit app ready to debug
</commit_message>
<xml_diff>
--- a/data/EN/cards_texts/black_cards.xlsx
+++ b/data/EN/cards_texts/black_cards.xlsx
@@ -1,553 +1,1069 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\!Master\Tesis\5 Codigo de Calidad P1\Cards_Against_AI\data\EN\cards_texts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Documents\!Master\Tesis\0 Datasets\decks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F947183C-BAF3-47B1-B562-F4C727142D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F244DF5-22D6-40C1-BD7F-0F7CB62628A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="texts" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="348">
+  <si>
+    <t>card_id</t>
+  </si>
+  <si>
+    <t>card_text</t>
+  </si>
   <si>
     <t>B001</t>
   </si>
   <si>
-    <t>It's a pity that kids these days are all getting involved with _______.</t>
+    <t>I like ______ and I cannot lie!</t>
   </si>
   <si>
     <t>B002</t>
   </si>
   <si>
-    <t>TFL apologizes for the delay in train service due to _______.</t>
+    <t>And the theme for this year’s winter formal is: “A Night of _____________.”</t>
   </si>
   <si>
     <t>B003</t>
   </si>
   <si>
-    <t>Do NOT go here! Found _______ in my spaghetti bolognese!</t>
+    <t>And today’s soup is Cream of _____________.</t>
   </si>
   <si>
     <t>B004</t>
   </si>
   <si>
-    <t>Nobody expects the Spanish Inquisition. Our chief weapons are fear, surprise, and _______.</t>
+    <t>B005</t>
+  </si>
+  <si>
+    <t>As your doctor, I must say this amount of _____________ is abnormal for a girl your age.</t>
   </si>
   <si>
     <t>B006</t>
   </si>
   <si>
-    <t>Military historians remember Alexander the Great for his brilliant use of _______ against the Persians.</t>
+    <t>Attention Target shoppers. Unfortunately, we will be closing early due to _____________.</t>
   </si>
   <si>
     <t>B007</t>
   </si>
   <si>
-    <t>What are my parents hiding from me? _______.</t>
+    <t>Boys love _____________.</t>
   </si>
   <si>
     <t>B008</t>
   </si>
   <si>
-    <t>Coming to the West End this year, _______: The Musical.</t>
+    <t>Come on guys! Let’s go downstairs and play my favorite game: _____________ in the Basement!</t>
   </si>
   <si>
     <t>B009</t>
   </si>
   <si>
-    <t>Life for American Indians was forever changed when the White Man introduced them to _______.</t>
+    <t>Darn kids! In my day, all we needed to have fun was _____________.</t>
   </si>
   <si>
     <t>B010</t>
   </si>
   <si>
-    <t>What's a girl's best friend? _______.</t>
+    <t>Designers! For this week’s challenge, you must make a dress designed for _____________.</t>
   </si>
   <si>
     <t>B011</t>
   </si>
   <si>
-    <t>Fun tip! When your man asks you to go down on him, try surprising him with _______ instead.</t>
+    <t>Do NOT go in the pool. There’s _____________ in there.</t>
   </si>
   <si>
     <t>B012</t>
   </si>
   <si>
-    <t>What is Batman's guilty pleasure? _______.</t>
+    <t>Holy crap! My video of _____________ has ten million views!</t>
   </si>
   <si>
     <t>B013</t>
   </si>
   <si>
-    <t>When Pharaoh remained unmoved, Moses called down a Plague of _______.</t>
+    <t>Easy or not, here comes _____________!</t>
   </si>
   <si>
     <t>B014</t>
   </si>
   <si>
-    <t>Airport security guidelines now prohibit _______ on airplanes.</t>
+    <t>Holy MOLY! Now THAT’S what I call _____________!</t>
   </si>
   <si>
     <t>B015</t>
   </si>
   <si>
-    <t>Once you pop, the fun don't stop! _______.</t>
+    <t>Honey, leave your sister alone. She’s busy with _____________.</t>
   </si>
   <si>
     <t>B016</t>
   </si>
   <si>
-    <t>That's why mums go to Iceland. _______.</t>
+    <t>I can show you _____________. Shining, shimmering, splendid.</t>
+  </si>
+  <si>
+    <t>B017</t>
+  </si>
+  <si>
+    <t>I have an extremely rare condition called “_____________ Face.”</t>
   </si>
   <si>
     <t>B018</t>
   </si>
   <si>
-    <t>What's my secret power? _______.</t>
+    <t>I put a spell on you! And now you’re _____________.</t>
   </si>
   <si>
     <t>B019</t>
   </si>
   <si>
-    <t>Daddy, why is mummy crying? _______.</t>
+    <t>If I had a million dollars, I’d spend it all on _____________.</t>
+  </si>
+  <si>
+    <t>B020</t>
+  </si>
+  <si>
+    <t>Listen! I’m from the future. You’ve got to stop _____________!</t>
   </si>
   <si>
     <t>B021</t>
   </si>
   <si>
-    <t>How did I lose my virginity? _______.</t>
+    <t>Mamma Mia. Here I go again. My my! How can I resist _____________?</t>
   </si>
   <si>
     <t>B022</t>
   </si>
   <si>
-    <t>White people like _______.</t>
+    <t>Next in the talent show, Jordan will wow us with _____________.</t>
   </si>
   <si>
     <t>B023</t>
   </si>
   <si>
-    <t>Here is the church. Here is the steeple. Open the doors, And there is _______.</t>
+    <t>Nothing brings a family together quite like _____________.</t>
   </si>
   <si>
     <t>B024</t>
   </si>
   <si>
-    <t>_______? Jim'll fix it!</t>
+    <t>Oh no. Mom’s new boyfriend is _____________.</t>
   </si>
   <si>
     <t>B025</t>
   </si>
   <si>
-    <t>Hey Reddit! I'm _______. Ask me anything.</t>
+    <t>Son, we need to talk. We found _____________ under your bed.</t>
   </si>
   <si>
     <t>B026</t>
   </si>
   <si>
-    <t>Next from J.K. Rowling: Harry Potter and the Chamber of _______.</t>
+    <t>Thanks for coming to babysit! Just a heads up: Kayla’s going through a bit of a “_____________” phase.</t>
   </si>
   <si>
     <t>B027</t>
   </si>
   <si>
-    <t>What made my first kiss so awkward? _______.</t>
+    <t>The President called. He needs _____________, NOW!</t>
   </si>
   <si>
     <t>B028</t>
   </si>
   <si>
-    <t>Uh, hey guys, I know this was my idea, but I'm having serious doubts about _______.</t>
+    <t>This election day, remember: a vote for me is a vote for _____________.</t>
   </si>
   <si>
     <t>B029</t>
   </si>
   <si>
-    <t>Why do I hurt all over? _______.</t>
+    <t>This is your captain speaking. Fasten your seatbelts and prepare for _____________.</t>
+  </si>
+  <si>
+    <t>B030</t>
+  </si>
+  <si>
+    <t>Today, we had a school assembly warning about the dangers of _____________.</t>
   </si>
   <si>
     <t>B031</t>
   </si>
   <si>
-    <t>I get by with a little help from _______.</t>
+    <t>We’re good, Mom! Other than _____________, we’re all good!</t>
   </si>
   <si>
     <t>B032</t>
   </si>
   <si>
-    <t>Next up on Channel 4: Ramsay's _______ Nightmares.</t>
+    <t>What ruined Christmas?_____________.</t>
   </si>
   <si>
     <t>B033</t>
   </si>
   <si>
-    <t>When I am Prime Minister of the United Kingdom, I will create the Ministry of _______.</t>
+    <t>Welcome to Kevin’s Pizza, where every pizza comes with _____________!</t>
   </si>
   <si>
     <t>B034</t>
   </si>
   <si>
-    <t>Dear Agony Aunt, I'm having some trouble with _______ and I need your advice.</t>
+    <t>What would be way cooler on fire?_____________.</t>
   </si>
   <si>
     <t>B035</t>
   </si>
   <si>
-    <t>Maybe she's born with it. Maybe it's _______.</t>
+    <t>What’s my superpower?_____________.</t>
   </si>
   <si>
     <t>B036</t>
   </si>
   <si>
-    <t>As the mum of five rambunctious boys, I'm no stranger to _______.</t>
+    <t>When I grow up, I’m gonna be _____________.</t>
   </si>
   <si>
     <t>B037</t>
   </si>
   <si>
-    <t>Why is Alan so sweaty? _______.</t>
+    <t>Yarrrr! Captain Jack, ’tis bad luck to bring _____________ aboard a ship!</t>
   </si>
   <si>
     <t>B038</t>
   </si>
   <si>
-    <t>UKIP: Putting _______ First!</t>
+    <t>According to a new report from the Pentagon, the greatest threat to national security is _______.</t>
   </si>
   <si>
     <t>B039</t>
   </si>
   <si>
-    <t>What will always get you laid? _______.</t>
+    <t>Alright! Answered two whole emails. Time to reward myself with _______.</t>
   </si>
   <si>
     <t>B040</t>
   </si>
   <si>
-    <t>What ended my last relationship? _______.</t>
+    <t>At our dojo, you’ll learn that your greatest weapon is not a punch or a kick. It’s _______.</t>
   </si>
   <si>
     <t>B041</t>
   </si>
   <si>
-    <t>Just once, I'd like to hear you say "Thanks, Mum. Thanks for _______."</t>
+    <t>Boomers love _______.</t>
   </si>
   <si>
     <t>B042</t>
   </si>
   <si>
-    <t>What's there a ton of in heaven? _______.</t>
+    <t>BREAKING NEWS: Elon Musk has acquired _______.</t>
   </si>
   <si>
     <t>B043</t>
   </si>
   <si>
+    <t>Cecilia! I’m down on my knees. I’m begging you please for _______.</t>
+  </si>
+  <si>
     <t>B044</t>
   </si>
   <si>
-    <t>When I am a billionaire, I shall erect a 50-foot statue to commemorate _______.</t>
+    <t>Congress has approved a $10 billion aid package to provide Ukraine with _______.</t>
+  </si>
+  <si>
+    <t>B045</t>
+  </si>
+  <si>
+    <t>Dear Diary: I met the cutest boy today. He has gorgeous blue eyes, and he loves_______, and that's what Ilike the must.</t>
   </si>
   <si>
     <t>B046</t>
   </si>
   <si>
-    <t>I got 99 problems but _______ ain't one.</t>
+    <t>God dammit! The wife’s complainin’ about _______ again.</t>
   </si>
   <si>
     <t>B047</t>
   </si>
   <si>
-    <t>Why am I sticky? _______.</t>
+    <t>Hello, I’m Mark Zuckerberg. Welcome to the Metaverse, where you can experience _______ like never before.</t>
   </si>
   <si>
     <t>B048</t>
   </si>
   <si>
-    <t>In Belmarsh Prison, word is you can trade 200 cigarettes for _______.</t>
+    <t>Hello, is this the front desk? Yeah, uh, I’m having a little trouble with _______ in my room.</t>
   </si>
   <si>
     <t>B049</t>
   </si>
   <si>
-    <t>Just saw this upsetting video! Please retweet!! #stop_______.</t>
+    <t>Hi, my name is Alex, and I’m an addict. It’s not the pills or the booze for me. It’s _______.</t>
+  </si>
+  <si>
+    <t>B050</t>
+  </si>
+  <si>
+    <t>Ho LAWD! All this _______ makin’ me sweat like a pig!</t>
   </si>
   <si>
     <t>B051</t>
   </si>
   <si>
-    <t>Alternative medicine is now embracing the curative powers of _______.</t>
+    <t>I don’t care what a guy looks like. As long as he’s _______, I’ll fuck him.</t>
   </si>
   <si>
     <t>B052</t>
   </si>
   <si>
-    <t>What makes life worth living? _______.</t>
+    <t>I swear, ladies, all the good men are either gay, taken, or _______.</t>
   </si>
   <si>
     <t>B053</t>
   </si>
   <si>
-    <t>What's the next Happy Meal® toy? _______.</t>
+    <t>I’d like to thank my husband, the cast and crew… but most importantly, I couldn’t have done it without _______!</t>
   </si>
   <si>
     <t>B054</t>
   </si>
   <si>
-    <t>Hey guys, welcome to TGI Fridays! Would you like to start the night off right with _______?</t>
+    <t>I’m afraid your college application needs some work. “_______” is not an extracurricular activity.</t>
   </si>
   <si>
     <t>B055</t>
   </si>
   <si>
-    <t>What's George W. Bush thinking about right now? _______.</t>
+    <t>I’m Kaylee, and welcome to my YouTube channel, “Mama Knows Best.” Follow me for more tips on _______!</t>
   </si>
   <si>
     <t>B056</t>
   </si>
   <si>
-    <t>_______: Kid-tested, mother-approved.</t>
+    <t>Kids grow up so fast! One day they’re learning to ride a bike, the next thing you know they’re _______.</t>
   </si>
   <si>
     <t>B057</t>
   </si>
   <si>
-    <t>It's a trap! _______</t>
+    <t>Ladies, if he doesn’t like _______, dump his ass!</t>
   </si>
   <si>
     <t>B058</t>
   </si>
   <si>
-    <t>If you can't be with the one you love, love _______.</t>
+    <t>My love language is _______.</t>
   </si>
   <si>
     <t>B059</t>
   </si>
   <si>
-    <t>The theme for next year's Eurovision Song Contest is "We are _______."</t>
+    <t>My wife and I saw you across the bar, and we love your vibe. Would you be interested in _______?</t>
   </si>
   <si>
     <t>B060</t>
   </si>
   <si>
-    <t>A romantic, candlelit dinner would be incomplete without _______.</t>
+    <t>Nah, man, I don’t fuck with _______.</t>
+  </si>
+  <si>
+    <t>B061</t>
+  </si>
+  <si>
+    <t>Okay, so…is it a red flag if your date just talks about _______ the whole time?</t>
   </si>
   <si>
     <t>B062</t>
   </si>
   <si>
-    <t>Now at the Natural History Museum: an interactive exhibit on _______.</t>
+    <t>Please, please support my friend Katie’s GoFundMe. She really needs money for _______.</t>
   </si>
   <si>
     <t>B063</t>
   </si>
   <si>
-    <t>Today on The Jeremy Kyle Show: "Help! My son is _______!"</t>
+    <t>So beautiful! Watch as this little boy with new cochlear implants hears _______ for the first time.</t>
   </si>
   <si>
     <t>B064</t>
   </si>
   <si>
-    <t>During sex, I like to think about _______.</t>
+    <t>Stop mom-shaming me! There’s nothing wrong with posting a pic of my kids enjoying _______.</t>
+  </si>
+  <si>
+    <t>B065</t>
+  </si>
+  <si>
+    <t>Subscribe to my OnlyFans for daily nudes and pictures of _______.</t>
+  </si>
+  <si>
+    <t>B066</t>
+  </si>
+  <si>
+    <t>Uncle Steve, this is a funeral. This is not the time for _______.</t>
   </si>
   <si>
     <t>B067</t>
   </si>
   <si>
-    <t>What would grandma find disturbing, yet oddly charming? _______.</t>
+    <t>Welcome to the WORLD’S SPOOKIEST Haunted House! We’ve got THRILLS! We’ve got CHILLS! We’ve got _______!</t>
   </si>
   <si>
     <t>B068</t>
   </si>
   <si>
-    <t>What's that sound? _______.</t>
+    <t>What’s actually slang for anal?______.</t>
   </si>
   <si>
     <t>B069</t>
   </si>
   <si>
-    <t>How am I maintaining my relationship status? _______.</t>
+    <t>______ is back! Only at McDonald’s.</t>
   </si>
   <si>
     <t>B070</t>
   </si>
   <si>
-    <t>I'm no doctor, but I'm pretty sure what you're suffering from is called "_______."</t>
+    <t>______. Awesome in theory, kind of a mess in practice.</t>
   </si>
   <si>
     <t>B071</t>
   </si>
   <si>
-    <t>What never fails to liven up the party? _______.</t>
+    <t>A remarkable new study has shown that chimps have evolved their own primitive version of ______.</t>
   </si>
   <si>
     <t>B072</t>
   </si>
   <si>
-    <t>War! What is it good for? _______.</t>
+    <t>And I would have gotten away with it, too, if it hadn’t been for ______!</t>
   </si>
   <si>
     <t>B073</t>
   </si>
   <si>
-    <t>This is the way the world ends. This is the way the world ends. Not with a bang but with _______.</t>
+    <t>And what did you bring for show and tell?______.</t>
   </si>
   <si>
     <t>B074</t>
   </si>
   <si>
-    <t>The school trip was completely ruined by _______.</t>
+    <t>As part of his daily regimen, Anderson Cooper sets aside 15 minutes for ______.</t>
   </si>
   <si>
     <t>B075</t>
   </si>
   <si>
-    <t>Instead of coal, Father Christmas now gives bad children _______.</t>
+    <t>Call the law offices of Goldstein &amp; Goldstein, because no one should have to tolerate ______ in the workplace.</t>
   </si>
   <si>
     <t>B076</t>
   </si>
   <si>
-    <t>Why can't I sleep at night? _______.</t>
+    <t>Charades were ruined for me forever when my mom had to act out ______.</t>
   </si>
   <si>
     <t>B077</t>
   </si>
   <si>
-    <t>Well if you'll excuse me, gentlemen, I have a date with _______.</t>
+    <t>Doctor, you’ve gone too far! The human body wasn’t meant to withstand that amount of ______!</t>
   </si>
   <si>
     <t>B078</t>
   </si>
   <si>
-    <t>Netflix's new reality show features twelve hot singles living with _______.</t>
+    <t>During high school I never really fit in until I found ______ club.</t>
   </si>
   <si>
     <t>B079</t>
   </si>
   <si>
-    <t>What gives me uncontrollable gas? _______.</t>
+    <t>During his midlife crisis, my dad got really into ______.</t>
   </si>
   <si>
     <t>B080</t>
   </si>
   <si>
-    <t>I'm sorry, Sir, but I couldn't complete my homework because of _______.</t>
+    <t>Finally! A service that delivers ______ right to your door.</t>
   </si>
   <si>
     <t>B081</t>
   </si>
   <si>
-    <t>This season at the Old Vic, Samuel Beckett's classic existential play, Waiting for _______.</t>
+    <t>Future Historians will agree that ______ marked the beginning of America’s decline.</t>
   </si>
   <si>
     <t>B082</t>
   </si>
   <si>
-    <t>That was so metal. _______</t>
+    <t>Hey baby, come back to my place and I’ll show you ______.</t>
+  </si>
+  <si>
+    <t>B083</t>
+  </si>
+  <si>
+    <t>I learned the hard way that you can’t cheer up a grieving friend with ______.</t>
+  </si>
+  <si>
+    <t>B084</t>
+  </si>
+  <si>
+    <t>I’m not like the rest of you. I’m too rich and busy for ______.</t>
   </si>
   <si>
     <t>B085</t>
   </si>
   <si>
-    <t>Mr. and Mrs. Diaz, we called you in because we're concerned about Cynthia. Are you aware that your daughter is _______?</t>
+    <t>In his new self-produced album, Kanye West raps over the sounds of ______.</t>
   </si>
   <si>
     <t>B086</t>
   </si>
   <si>
-    <t>I drink to forget _______.</t>
+    <t>In his newest and most difficult stunt, David Blaine must escape from ______.</t>
   </si>
   <si>
     <t>B087</t>
   </si>
   <si>
-    <t>Next on Sky Sports: The World Championship of _______.</t>
-  </si>
-  <si>
-    <t>But before I kill you, Mr. Bond, I must show you _______.</t>
-  </si>
-  <si>
-    <t>Check me out, yo! I call this dance move "_______."</t>
-  </si>
-  <si>
-    <t>Old MacDonald had _______. E-I-E-I-O.</t>
-  </si>
-  <si>
-    <t>What's that smell? _______.</t>
-  </si>
-  <si>
-    <t>Kids, I don't need drugs to get high. I'm on high on _______.</t>
-  </si>
-  <si>
-    <t>What did I bring back from Amsterdam? _______.</t>
-  </si>
-  <si>
-    <t>A recent laboratory study shows that undergraduates have 50% less sex after being exposed to _______.</t>
-  </si>
-  <si>
-    <t>After four platinum albums and three Grammys, it's time to get back to my roots, to what inspired me to make music in the first place: _______.</t>
-  </si>
-  <si>
-    <t>Mate, do not go in that bathroom. There's _______ in there.</t>
-  </si>
-  <si>
-    <t>50% of all marriages end in _______.</t>
-  </si>
-  <si>
-    <t>I'm going on a cleanse this week. Nothing but kale juice and _______.</t>
-  </si>
-  <si>
-    <t>Click Here For _______!!!</t>
-  </si>
-  <si>
-    <t>card_text</t>
-  </si>
-  <si>
-    <t>B005</t>
-  </si>
-  <si>
-    <t>B017</t>
-  </si>
-  <si>
-    <t>B020</t>
-  </si>
-  <si>
-    <t>B030</t>
-  </si>
-  <si>
-    <t>B045</t>
-  </si>
-  <si>
-    <t>B050</t>
-  </si>
-  <si>
-    <t>B061</t>
-  </si>
-  <si>
-    <t>B065</t>
-  </si>
-  <si>
-    <t>B066</t>
-  </si>
-  <si>
-    <t>B083</t>
-  </si>
-  <si>
-    <t>B084</t>
-  </si>
-  <si>
-    <t>card_id</t>
+    <t>In its new tourism campaign, Detroit proudly proclaims that it has finally eliminated ______.</t>
+  </si>
+  <si>
+    <t>B088</t>
+  </si>
+  <si>
+    <t>In the seventh circle of Hell, sinners must endure ______ for all eternity.</t>
+  </si>
+  <si>
+    <t>B089</t>
+  </si>
+  <si>
+    <t>Legend has it Prince wouldn’t perform without ______ in his dressing room.</t>
+  </si>
+  <si>
+    <t>B090</t>
+  </si>
+  <si>
+    <t>Little Miss Muffet Sat on a tuffet, Eating her curds and ______.</t>
+  </si>
+  <si>
+    <t>B091</t>
+  </si>
+  <si>
+    <t>Lovin’ you is easy ’cause you’re ______.</t>
+  </si>
+  <si>
+    <t>B092</t>
+  </si>
+  <si>
+    <t>Members of New York’s social elite are paying thousands of dollars just to experience ______.</t>
+  </si>
+  <si>
+    <t>B093</t>
+  </si>
+  <si>
+    <t>Money can’t buy me love, but it can buy me ______.</t>
+  </si>
+  <si>
+    <t>B094</t>
+  </si>
+  <si>
+    <t>My country, ’tis of thee, sweet land of ______.</t>
+  </si>
+  <si>
+    <t>B095</t>
+  </si>
+  <si>
+    <t>My gym teacher got fired for adding ______ to the obstacle course.</t>
+  </si>
+  <si>
+    <t>B096</t>
+  </si>
+  <si>
+    <t>My plan for world domination begins with ______.</t>
+  </si>
+  <si>
+    <t>B097</t>
+  </si>
+  <si>
+    <t>Next time on Dr. Phil: How to talk to your child about ______.</t>
+  </si>
+  <si>
+    <t>B098</t>
+  </si>
+  <si>
+    <t>Next week on the Discovery Channel, one man must survive in the depths of the Amazon with only ______ and his wits.</t>
+  </si>
+  <si>
+    <t>B099</t>
+  </si>
+  <si>
+    <t>Only two things in life are certain: death and ______.</t>
+  </si>
+  <si>
+    <t>B100</t>
+  </si>
+  <si>
+    <t>Science will never explain ______.</t>
+  </si>
+  <si>
+    <t>B101</t>
+  </si>
+  <si>
+    <t>The blind date was going horribly until we discovered our shared interest in ______.</t>
+  </si>
+  <si>
+    <t>B102</t>
+  </si>
+  <si>
+    <t>The healing process began when I joined a support group for victims of ______.</t>
+  </si>
+  <si>
+    <t>B103</t>
+  </si>
+  <si>
+    <t>The secret to a lasting marriage is communication, communication, and ______.</t>
+  </si>
+  <si>
+    <t>B104</t>
+  </si>
+  <si>
+    <t>This month’s Cosmo: “Spice up your sex life by bringing ______ into the bedroom.”</t>
+  </si>
+  <si>
+    <t>B105</t>
+  </si>
+  <si>
+    <t>To prepare for his upcoming role, Daniel Day-Lewis immersed himself in the world of ______.</t>
+  </si>
+  <si>
+    <t>B106</t>
+  </si>
+  <si>
+    <t>Tonight on 20/20: What you don’t know about ______ could kill you.</t>
+  </si>
+  <si>
+    <t>B107</t>
+  </si>
+  <si>
+    <t>Welcome to Señor Frog’s! Would you like to try our signature cocktail, “______ on the Beach”?</t>
+  </si>
+  <si>
+    <t>B108</t>
+  </si>
+  <si>
+    <t>What brought the orgy to a grinding halt?______.</t>
+  </si>
+  <si>
+    <t>B109</t>
+  </si>
+  <si>
+    <t>What left this stain on my couch?______.</t>
+  </si>
+  <si>
+    <t>B110</t>
+  </si>
+  <si>
+    <t>What makes Grandma feel young again?______.</t>
+  </si>
+  <si>
+    <t>B111</t>
+  </si>
+  <si>
+    <t>What makes me cry every time?______.</t>
+  </si>
+  <si>
+    <t>B112</t>
+  </si>
+  <si>
+    <t>When all else fails, I can always masturbate to ______.</t>
+  </si>
+  <si>
+    <t>B113</t>
+  </si>
+  <si>
+    <t>When I pooped, what came out of my butt?______.</t>
+  </si>
+  <si>
+    <t>B114</t>
+  </si>
+  <si>
+    <t>When the dog bites / When the bee stings / When I’m feeling sad / I simply remember ______ / And then I don’t feel so bad.</t>
+  </si>
+  <si>
+    <t>B115</t>
+  </si>
+  <si>
+    <t>Your persistence is admirable, my dear Prince. But you cannot win my heart with ______ alone.</t>
+  </si>
+  <si>
+    <t>B116</t>
+  </si>
+  <si>
+    <t>Believe it or not, Jim Carrey can do a dead-on impression of ______.</t>
+  </si>
+  <si>
+    <t>B117</t>
+  </si>
+  <si>
+    <t>How did Stella get her groove back?______.</t>
+  </si>
+  <si>
+    <t>B118</t>
+  </si>
+  <si>
+    <t>B119</t>
+  </si>
+  <si>
+    <t>I’m a bitch, I’m a lover, I’m a child, I’m ______.</t>
+  </si>
+  <si>
+    <t>B120</t>
+  </si>
+  <si>
+    <t>Siskel and Ebert have panned ______ as “poorly conceived” and “sloppily executed.”</t>
+  </si>
+  <si>
+    <t>B121</t>
+  </si>
+  <si>
+    <t>Tonight on SNICK: “Are You Afraid of ______?</t>
+  </si>
+  <si>
+    <t>B122</t>
+  </si>
+  <si>
+    <t>Up next on Nickelodeon: “Clarissa Explains ______.”</t>
+  </si>
+  <si>
+    <t>B123</t>
+  </si>
+  <si>
+    <t>______? That’s a no from me, dawg.</t>
+  </si>
+  <si>
+    <t>B124</t>
+  </si>
+  <si>
+    <t>B125</t>
+  </si>
+  <si>
+    <t>I couldn’t help but wonder. Was “having it all” an unattainable myth? Was the secret to a truly happy life just ______?</t>
+  </si>
+  <si>
+    <t>B126</t>
+  </si>
+  <si>
+    <t>Oh my god! ______ killed Kenny!</t>
+  </si>
+  <si>
+    <t>B127</t>
+  </si>
+  <si>
+    <t>Oops! I did it again. I played with ______.</t>
+  </si>
+  <si>
+    <t>B128</t>
+  </si>
+  <si>
+    <t>“They’re bringing drugs. They’re bringing crime. They’re rapists. I assume, they are _____.”</t>
+  </si>
+  <si>
+    <t>B129</t>
+  </si>
+  <si>
+    <t>Oh shit! I just got ______.</t>
+  </si>
+  <si>
+    <t>B130</t>
+  </si>
+  <si>
+    <t>The fault, dear Brutus, is not in our stars, but in ______.</t>
+  </si>
+  <si>
+    <t>B131</t>
+  </si>
+  <si>
+    <t>We want a pitcher, not ______!</t>
+  </si>
+  <si>
+    <t>B132</t>
+  </si>
+  <si>
+    <t>When asked about the biggest threat facing the nation, 60% of Americans said ______.</t>
+  </si>
+  <si>
+    <t>B133</t>
+  </si>
+  <si>
+    <t>You see, son, baseball is like ______. Don’t overthink it.</t>
+  </si>
+  <si>
+    <t>B134</t>
+  </si>
+  <si>
+    <t>Everyone is staring at you because you’re ___.</t>
+  </si>
+  <si>
+    <t>B135</t>
+  </si>
+  <si>
+    <t>Hold up. I gotta deal with ___, then l’mma smoke this.</t>
+  </si>
+  <si>
+    <t>B136</t>
+  </si>
+  <si>
+    <t>Okay here’s the pitch. James Franco and Seth Rogen are trying to score some weed, and then ___ happens.</t>
+  </si>
+  <si>
+    <t>B137</t>
+  </si>
+  <si>
+    <t>You know what’s, like, really funny when you think about it? ___.</t>
+  </si>
+  <si>
+    <t>______: The reason why the world is full of famine and AIDS.</t>
+  </si>
+  <si>
+    <t>Killing  ____ in the middle of a civil rights march.</t>
+  </si>
+  <si>
+    <t>Stealing jobs and raping your daughters, that's what ______ means.</t>
+  </si>
+  <si>
+    <t>____: bringing gifts to ghettos full of criminals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ____: Eating dogs and smelling like rancid fish.</t>
+  </si>
+  <si>
+    <t>____ so that illegals stay and vote for Democrats.</t>
+  </si>
+  <si>
+    <t>____: the only place where blacks don't steal chicken.</t>
+  </si>
+  <si>
+    <t>Eternal hatred towards ____ and its social parasitism.</t>
+  </si>
+  <si>
+    <t>____: yellow savages who conquered Asia with mass rapes.</t>
+  </si>
+  <si>
+    <t>Training ____ to bite all non-whites.</t>
+  </si>
+  <si>
+    <t>Yelling ____ while lynching a black person.</t>
+  </si>
+  <si>
+    <t>I saw ____ shitting themselves with fear at the migrant invasion.</t>
+  </si>
+  <si>
+    <t>Is that poop or just ____ trying to integrate?</t>
+  </si>
+  <si>
+    <t>____: the subsidy for immigrants layabouts.</t>
+  </si>
+  <si>
+    <t>____is fucking your wife while you work double shifts.</t>
+  </si>
+  <si>
+    <t>____, valid excuse for crime, drugs, and eternal complaining.</t>
+  </si>
+  <si>
+    <t>____: the only unforgivable sin in the woke agenda.</t>
+  </si>
+  <si>
+    <t>____is destroying white economies.</t>
+  </si>
+  <si>
+    <t>What do you like most in life? ____ .</t>
+  </si>
+  <si>
+    <t>____: the only smart way to avoid terrorists.</t>
+  </si>
+  <si>
+    <t>____: blond traitors committing suicide with immigration.</t>
+  </si>
+  <si>
+    <t>____, the white genocide.</t>
+  </si>
+  <si>
+    <t>Superior, but guilty for existing: ____.</t>
+  </si>
+  <si>
+    <t>____: the best solution to any problem.</t>
+  </si>
+  <si>
+    <t>____: every American patriot's wet dream.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mexicans showed us _______. </t>
+  </si>
+  <si>
+    <t>____ from the cradle to save the race.</t>
+  </si>
+  <si>
+    <t>Sometimes I have nightmares about _________.</t>
+  </si>
+  <si>
+    <t>Arriving in hell you encounter: _______.</t>
+  </si>
+  <si>
+    <t>Germans' favorite toys: ____.</t>
+  </si>
+  <si>
+    <t>Moving to China so I don't have to see ____.</t>
+  </si>
+  <si>
+    <t>It's incredible how much ____ there can be</t>
+  </si>
+  <si>
+    <t>Having ____ in the country lowers our quality of life.</t>
+  </si>
+  <si>
+    <t>It is impossible for ____ to stay at home.</t>
+  </si>
+  <si>
+    <t>My mom punished me by not letting me leave the house for a week because I was bringing _____ home.</t>
+  </si>
+  <si>
+    <t>____: the ultimate hate crime.</t>
+  </si>
+  <si>
+    <t>B138</t>
+  </si>
+  <si>
+    <t>B139</t>
+  </si>
+  <si>
+    <t>B140</t>
+  </si>
+  <si>
+    <t>B141</t>
+  </si>
+  <si>
+    <t>B142</t>
+  </si>
+  <si>
+    <t>B143</t>
+  </si>
+  <si>
+    <t>B144</t>
+  </si>
+  <si>
+    <t>B145</t>
+  </si>
+  <si>
+    <t>B146</t>
+  </si>
+  <si>
+    <t>B147</t>
+  </si>
+  <si>
+    <t>B148</t>
+  </si>
+  <si>
+    <t>B149</t>
+  </si>
+  <si>
+    <t>B150</t>
+  </si>
+  <si>
+    <t>B151</t>
+  </si>
+  <si>
+    <t>B152</t>
+  </si>
+  <si>
+    <t>B153</t>
+  </si>
+  <si>
+    <t>B154</t>
+  </si>
+  <si>
+    <t>B155</t>
+  </si>
+  <si>
+    <t>B156</t>
+  </si>
+  <si>
+    <t>B157</t>
+  </si>
+  <si>
+    <t>B158</t>
+  </si>
+  <si>
+    <t>B159</t>
+  </si>
+  <si>
+    <t>B160</t>
+  </si>
+  <si>
+    <t>B161</t>
+  </si>
+  <si>
+    <t>B162</t>
+  </si>
+  <si>
+    <t>B163</t>
+  </si>
+  <si>
+    <t>B164</t>
+  </si>
+  <si>
+    <t>B165</t>
+  </si>
+  <si>
+    <t>B166</t>
+  </si>
+  <si>
+    <t>B167</t>
+  </si>
+  <si>
+    <t>B168</t>
+  </si>
+  <si>
+    <t>B169</t>
+  </si>
+  <si>
+    <t>B170</t>
+  </si>
+  <si>
+    <t>B171</t>
+  </si>
+  <si>
+    <t>B172</t>
+  </si>
+  <si>
+    <t>B173</t>
+  </si>
+  <si>
+    <t>100 people. 39 days of ______. One Survivor.</t>
+  </si>
+  <si>
+    <t>____: the perfect duo to destroy any country.</t>
+  </si>
+  <si>
+    <t>Anyone can dance! Just throw your hands in the air and pretend you’re _____________!</t>
   </si>
 </sst>
 </file>
@@ -574,12 +1090,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -609,11 +1131,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -916,327 +1439,327 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B88"/>
+  <dimension ref="A1:B174"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="83.6640625" customWidth="1"/>
+    <col min="2" max="2" width="87.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>163</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>347</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="B17" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>165</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>166</v>
+        <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="B24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="B25" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B30" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>167</v>
+        <v>59</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B32" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="B39" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
         <v>78</v>
@@ -1244,7 +1767,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
         <v>80</v>
@@ -1252,7 +1775,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
         <v>82</v>
@@ -1260,7 +1783,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="B43" t="s">
         <v>84</v>
@@ -1268,7 +1791,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B44" t="s">
         <v>86</v>
@@ -1276,7 +1799,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
         <v>88</v>
@@ -1284,7 +1807,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>168</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
         <v>90</v>
@@ -1292,7 +1815,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
         <v>92</v>
@@ -1300,7 +1823,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>93</v>
       </c>
       <c r="B48" t="s">
         <v>94</v>
@@ -1308,7 +1831,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="B49" t="s">
         <v>96</v>
@@ -1316,7 +1839,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="B50" t="s">
         <v>98</v>
@@ -1324,7 +1847,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>169</v>
+        <v>99</v>
       </c>
       <c r="B51" t="s">
         <v>100</v>
@@ -1332,7 +1855,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="B52" t="s">
         <v>102</v>
@@ -1340,7 +1863,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s">
         <v>104</v>
@@ -1348,7 +1871,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="B54" t="s">
         <v>106</v>
@@ -1356,7 +1879,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="B55" t="s">
         <v>108</v>
@@ -1364,7 +1887,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="B56" t="s">
         <v>110</v>
@@ -1372,7 +1895,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="B57" t="s">
         <v>112</v>
@@ -1380,7 +1903,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="B58" t="s">
         <v>114</v>
@@ -1388,7 +1911,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="B59" t="s">
         <v>116</v>
@@ -1396,7 +1919,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="B60" t="s">
         <v>118</v>
@@ -1404,7 +1927,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="B61" t="s">
         <v>120</v>
@@ -1412,7 +1935,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>170</v>
+        <v>121</v>
       </c>
       <c r="B62" t="s">
         <v>122</v>
@@ -1420,7 +1943,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="B63" t="s">
         <v>124</v>
@@ -1428,7 +1951,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="B64" t="s">
         <v>126</v>
@@ -1436,7 +1959,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="B65" t="s">
         <v>128</v>
@@ -1444,7 +1967,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>171</v>
+        <v>129</v>
       </c>
       <c r="B66" t="s">
         <v>130</v>
@@ -1452,7 +1975,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
       <c r="B67" t="s">
         <v>132</v>
@@ -1460,7 +1983,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>113</v>
+        <v>133</v>
       </c>
       <c r="B68" t="s">
         <v>134</v>
@@ -1468,7 +1991,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="B69" t="s">
         <v>136</v>
@@ -1476,7 +1999,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>117</v>
+        <v>137</v>
       </c>
       <c r="B70" t="s">
         <v>138</v>
@@ -1484,7 +2007,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>119</v>
+        <v>139</v>
       </c>
       <c r="B71" t="s">
         <v>140</v>
@@ -1492,7 +2015,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="B72" t="s">
         <v>142</v>
@@ -1500,7 +2023,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>143</v>
       </c>
       <c r="B73" t="s">
         <v>144</v>
@@ -1508,7 +2031,7 @@
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="B74" t="s">
         <v>146</v>
@@ -1516,7 +2039,7 @@
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="B75" t="s">
         <v>148</v>
@@ -1524,7 +2047,7 @@
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="B76" t="s">
         <v>150</v>
@@ -1532,98 +2055,786 @@
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>131</v>
+        <v>151</v>
       </c>
       <c r="B77" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>133</v>
+        <v>153</v>
       </c>
       <c r="B78" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="B79" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="B80" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>139</v>
+        <v>159</v>
       </c>
       <c r="B81" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="B82" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>143</v>
+        <v>163</v>
       </c>
       <c r="B83" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="B84" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="B85" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B86" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="B87" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="B88" t="s">
-        <v>162</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>175</v>
+      </c>
+      <c r="B89" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>177</v>
+      </c>
+      <c r="B90" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>179</v>
+      </c>
+      <c r="B91" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>181</v>
+      </c>
+      <c r="B92" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>183</v>
+      </c>
+      <c r="B93" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>185</v>
+      </c>
+      <c r="B94" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>187</v>
+      </c>
+      <c r="B95" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>189</v>
+      </c>
+      <c r="B96" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>191</v>
+      </c>
+      <c r="B97" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>193</v>
+      </c>
+      <c r="B98" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>195</v>
+      </c>
+      <c r="B99" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>197</v>
+      </c>
+      <c r="B100" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>199</v>
+      </c>
+      <c r="B101" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>201</v>
+      </c>
+      <c r="B102" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>203</v>
+      </c>
+      <c r="B103" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>205</v>
+      </c>
+      <c r="B104" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>207</v>
+      </c>
+      <c r="B105" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>209</v>
+      </c>
+      <c r="B106" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>211</v>
+      </c>
+      <c r="B107" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>213</v>
+      </c>
+      <c r="B108" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>215</v>
+      </c>
+      <c r="B109" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>217</v>
+      </c>
+      <c r="B110" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>219</v>
+      </c>
+      <c r="B111" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>221</v>
+      </c>
+      <c r="B112" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>223</v>
+      </c>
+      <c r="B113" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>225</v>
+      </c>
+      <c r="B114" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>227</v>
+      </c>
+      <c r="B115" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>229</v>
+      </c>
+      <c r="B116" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>231</v>
+      </c>
+      <c r="B117" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>233</v>
+      </c>
+      <c r="B118" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>235</v>
+      </c>
+      <c r="B119" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>236</v>
+      </c>
+      <c r="B120" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>238</v>
+      </c>
+      <c r="B121" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>240</v>
+      </c>
+      <c r="B122" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>242</v>
+      </c>
+      <c r="B123" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>244</v>
+      </c>
+      <c r="B124" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>246</v>
+      </c>
+      <c r="B125" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>247</v>
+      </c>
+      <c r="B126" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>249</v>
+      </c>
+      <c r="B127" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>251</v>
+      </c>
+      <c r="B128" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>253</v>
+      </c>
+      <c r="B129" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>255</v>
+      </c>
+      <c r="B130" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>257</v>
+      </c>
+      <c r="B131" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>259</v>
+      </c>
+      <c r="B132" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>261</v>
+      </c>
+      <c r="B133" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>263</v>
+      </c>
+      <c r="B134" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>265</v>
+      </c>
+      <c r="B135" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>267</v>
+      </c>
+      <c r="B136" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>269</v>
+      </c>
+      <c r="B137" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>271</v>
+      </c>
+      <c r="B138" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>309</v>
+      </c>
+      <c r="B139" s="2" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>310</v>
+      </c>
+      <c r="B140" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>311</v>
+      </c>
+      <c r="B141" s="2" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>312</v>
+      </c>
+      <c r="B142" s="2" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>313</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>314</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>315</v>
+      </c>
+      <c r="B145" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>316</v>
+      </c>
+      <c r="B146" s="2" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>317</v>
+      </c>
+      <c r="B147" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>318</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>319</v>
+      </c>
+      <c r="B149" s="2" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>320</v>
+      </c>
+      <c r="B150" s="2" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>321</v>
+      </c>
+      <c r="B151" s="2" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>322</v>
+      </c>
+      <c r="B152" s="2" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>323</v>
+      </c>
+      <c r="B153" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>324</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>325</v>
+      </c>
+      <c r="B155" s="2" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>326</v>
+      </c>
+      <c r="B156" s="2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>327</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>328</v>
+      </c>
+      <c r="B158" s="2" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>329</v>
+      </c>
+      <c r="B159" s="2" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>330</v>
+      </c>
+      <c r="B160" s="2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>331</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>332</v>
+      </c>
+      <c r="B162" s="2" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>333</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>334</v>
+      </c>
+      <c r="B164" s="2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>335</v>
+      </c>
+      <c r="B165" s="2" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>336</v>
+      </c>
+      <c r="B166" s="2" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>337</v>
+      </c>
+      <c r="B167" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>338</v>
+      </c>
+      <c r="B168" s="2" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>339</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>340</v>
+      </c>
+      <c r="B170" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>341</v>
+      </c>
+      <c r="B171" s="2" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>342</v>
+      </c>
+      <c r="B172" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>343</v>
+      </c>
+      <c r="B173" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>344</v>
+      </c>
+      <c r="B174" t="s">
+        <v>308</v>
       </c>
     </row>
   </sheetData>

</xml_diff>